<commit_message>
Add daily checklist + launch-budget template to manager playbook
Sheet 6: one-page daily checklist (morning checks, threshold actions,
weekly tasks). Sheet 7: launch-budget calculator with live formulas
(inputs: margin, target/day, CPO start/target, weeks -> week-by-week
ramp, weekly profit, cumulative investment, break-even) + booster example.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0153XBqtvJYtRAKHdw3RmMsz
</commit_message>
<xml_diff>
--- a/outputs/ozon_ads/ozon_ad_manager_playbook_2026-10-05.xlsx
+++ b/outputs/ozon_ads/ozon_ad_manager_playbook_2026-10-05.xlsx
@@ -12,6 +12,8 @@
     <sheet name="3. Бюджет на вывод" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="4. Ежедневные правила" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="5. Метрики" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="6. Чек-лист (каждый день)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="7. Бюджет вывода (шаблон)" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47,7 +49,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -79,6 +81,11 @@
         <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2A8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -106,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -152,6 +159,22 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1424,4 +1447,505 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ЧЕК-ЛИСТ МЕНЕДЖЕРА — КАЖДЫЙ ДЕНЬ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>УТРО — проверить по каждой активной кампании:</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>☐ ДРР за вчера — в норме? (зрелый товар ≤15%, новый — ПАДАЕТ ли день ото дня)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>☐ CPO &lt; маржи/шт? Если выше — снизить ставку или пауза.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>☐ Есть ли сток по товару? Ушёл в 0 → поставить рекламу на паузу.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>☐ Нет ли кампаний, где бюджет растёт, а продажи/ДРР не улучшаются? → резать.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>ДЕЙСТВИЯ ПО ПОРОГАМ:</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>🟢 ДРР ≤10% и CPO &lt; маржи → поднять дневной бюджет на 20–30%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>🟡 ДРР 15–25% → снизить ставку; проверить сток/доставку (часто причина тут).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>🔴 ДРР &gt;25% или CPO &gt; маржи или клик→заказ &lt;2% → выключить/резать.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>🆕 Новый товар: ДРР высокий, но падает → продолжать вывод. Не падает 2–3 нед → стоп.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>РАЗ В НЕДЕЛЮ:</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>☐ Выгрузить статистику кампаний → таблица расход/ДРР/CPO по каждой.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>☐ Бюджет перекладывать: из убыточных (высокий ДРР) в прибыльные (ДРР ≤10%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>☐ Проверить позиции по главным ключам и отзывы у героев.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>☐ Запустить/проверить ретаргет по сегментам (кто смотрел/корзина) — после наличия стока.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>☐ Зайти в акции Ozon по ходовым товарам.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>ЗАПОМНИТЬ: главный закон — CPO &lt; маржи/шт. Реклама только на карточки со стоком. Бюджет — в поиск, не в холодные рекомендации.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A22:D23"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A13:D13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>РАСЧЁТ БЮДЖЕТА ВЫВОДА НОВОГО ТОВАРА (пример + шаблон)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>ВВОДНЫЕ (жёлтые — подставить свои):</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Товар (пример)</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>Celimax Pore+Dark пэды</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Маржа до рекламы, ₽/шт</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>450</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Цель продаж к концу вывода, шт/день</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>CPO на старте, ₽</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>CPO цель (зрелый), ₽</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Срок вывода, недель</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>ПЛАН ПО НЕДЕЛЯМ (считается автоматически):</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Неделя</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Продаж/день</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>CPO, ₽</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>ДРР примерно</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Расход/нед, ₽</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Прибыль/нед, ₽</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Накоплено прибыли, ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>1 (вывод)</t>
+        </is>
+      </c>
+      <c r="B13" s="6">
+        <f>ROUND($B$6*0.4,0)</f>
+        <v/>
+      </c>
+      <c r="C13" s="6">
+        <f>ROUND($B$8+($B$7-$B$8)*1.0,0)</f>
+        <v/>
+      </c>
+      <c r="D13" s="6">
+        <f>TEXT(C13/($B$5+C13)*100,"0")&amp;"%"</f>
+        <v/>
+      </c>
+      <c r="E13" s="7">
+        <f>ROUND(B13*C13*7,0)</f>
+        <v/>
+      </c>
+      <c r="F13" s="7">
+        <f>ROUND(B13*($B$5-C13)*7,0)</f>
+        <v/>
+      </c>
+      <c r="G13" s="7">
+        <f>F13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>2 (дозревание)</t>
+        </is>
+      </c>
+      <c r="B14" s="6">
+        <f>ROUND($B$6*0.7,0)</f>
+        <v/>
+      </c>
+      <c r="C14" s="6">
+        <f>ROUND($B$8+($B$7-$B$8)*0.5,0)</f>
+        <v/>
+      </c>
+      <c r="D14" s="6">
+        <f>TEXT(C14/($B$5+C14)*100,"0")&amp;"%"</f>
+        <v/>
+      </c>
+      <c r="E14" s="7">
+        <f>ROUND(B14*C14*7,0)</f>
+        <v/>
+      </c>
+      <c r="F14" s="7">
+        <f>ROUND(B14*($B$5-C14)*7,0)</f>
+        <v/>
+      </c>
+      <c r="G14" s="7">
+        <f>G13+F14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>3 (выход в плюс)</t>
+        </is>
+      </c>
+      <c r="B15" s="6">
+        <f>ROUND($B$6*1.0,0)</f>
+        <v/>
+      </c>
+      <c r="C15" s="6">
+        <f>ROUND($B$8+($B$7-$B$8)*0.15,0)</f>
+        <v/>
+      </c>
+      <c r="D15" s="6">
+        <f>TEXT(C15/($B$5+C15)*100,"0")&amp;"%"</f>
+        <v/>
+      </c>
+      <c r="E15" s="7">
+        <f>ROUND(B15*C15*7,0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="7">
+        <f>ROUND(B15*($B$5-C15)*7,0)</f>
+        <v/>
+      </c>
+      <c r="G15" s="7">
+        <f>G14+F15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>4 (заработок)</t>
+        </is>
+      </c>
+      <c r="B16" s="6">
+        <f>ROUND($B$6*1.1,0)</f>
+        <v/>
+      </c>
+      <c r="C16" s="6">
+        <f>ROUND($B$8+($B$7-$B$8)*0.0,0)</f>
+        <v/>
+      </c>
+      <c r="D16" s="6">
+        <f>TEXT(C16/($B$5+C16)*100,"0")&amp;"%"</f>
+        <v/>
+      </c>
+      <c r="E16" s="7">
+        <f>ROUND(B16*C16*7,0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="7">
+        <f>ROUND(B16*($B$5-C16)*7,0)</f>
+        <v/>
+      </c>
+      <c r="G16" s="7">
+        <f>G15+F16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>КАК ЧИТАТЬ:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>• Неделя 1 — «прибыль/нед» отрицательная: CPO выше маржи, это ИНВЕСТИЦИЯ в вывод (покупаешь позиции и отзывы).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>• По мере дозревания CPO падает → с 2–3 недели выходишь в плюс.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>• «Накоплено прибыли» — когда станет положительным, вывод окупился.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>• Бюджет на вывод = максимальный минус в колонке «Накоплено» (сколько денег нужно вложить, пока не окупится).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>• Если по факту CPO НЕ падает к цели за срок вывода — товар/канал не выводится, стоп (как рекомендации крем-бустера).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>ПРИМЕР КРЕМ-БУСТЕРА (факт): вкладывали ~50 тыс.₽/день, 2 недели ДРР падал 19%→7%, вывод удался — теперь зарабатывает ~200 ₽ с заказа × 150–185 заказов/день.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A23:G23"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>